<commit_message>
implemented progression and log scrapping, routes and Mainmenu and login
</commit_message>
<xml_diff>
--- a/webscrapping/sofascore/Server/files_initted/estadios_info_db.xlsx
+++ b/webscrapping/sofascore/Server/files_initted/estadios_info_db.xlsx
@@ -1,37 +1,132 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+  <si>
+    <t>id_estadio</t>
+  </si>
+  <si>
+    <t>nombre</t>
+  </si>
+  <si>
+    <t>latitud</t>
+  </si>
+  <si>
+    <t>longitud</t>
+  </si>
+  <si>
+    <t>capacidad</t>
+  </si>
+  <si>
+    <t>id_equipo</t>
+  </si>
+  <si>
+    <t>Estadi Montilivi</t>
+  </si>
+  <si>
+    <t>Estadio de la Ceramica</t>
+  </si>
+  <si>
+    <t>Estadi de Son Moix</t>
+  </si>
+  <si>
+    <t>Estadio de Mendizorroza</t>
+  </si>
+  <si>
+    <t>Mestalla</t>
+  </si>
+  <si>
+    <t>Estadio Abanca Balaídos</t>
+  </si>
+  <si>
+    <t>San Mamés</t>
+  </si>
+  <si>
+    <t>RCDE Stadium</t>
+  </si>
+  <si>
+    <t>Estadio Martínez Valero</t>
+  </si>
+  <si>
+    <t>Bernabéu</t>
+  </si>
+  <si>
+    <t>Benito Villamarin</t>
+  </si>
+  <si>
+    <t>Riyadh Air Metropolitano</t>
+  </si>
+  <si>
+    <t>Ciudad de Valencia</t>
+  </si>
+  <si>
+    <t>Estadio El Sadar</t>
+  </si>
+  <si>
+    <t>Reale Arena</t>
+  </si>
+  <si>
+    <t>Carlos Tartiere</t>
+  </si>
+  <si>
+    <t>Ramón Sánchez Pizjuán</t>
+  </si>
+  <si>
+    <t>Estadio de Vallecas</t>
+  </si>
+  <si>
+    <t>Coliseum Alfonso Pérez</t>
+  </si>
+  <si>
+    <t>Estadi Johan Cruyff</t>
+  </si>
+  <si>
+    <t>Olímpic Lluís Companys</t>
+  </si>
+  <si>
+    <t>Estadio de la Cartuja</t>
+  </si>
+  <si>
+    <t>Spotify Camp Nou</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,93 +141,35 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -420,553 +457,491 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>id_estadio</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>nombre</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>latitud</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>longitud</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>capacidad</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>id_equipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2">
         <v>260827297577701</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Estadi Montilivi</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2">
         <v>41.9611</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>2.8278</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>14624</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>24264</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
+    <row r="3" spans="1:6">
+      <c r="A3">
         <v>190203353926090</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Estadio de la Ceramica</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3">
         <v>39.944208</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3">
         <v>-0.103405</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>23500</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3">
         <v>2819</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="n">
+    <row r="4" spans="1:6">
+      <c r="A4">
         <v>99680602019422</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Estadi de Son Moix</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4">
         <v>39.589935</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4">
         <v>2.630116</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4">
         <v>26020</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4">
         <v>2826</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="n">
+    <row r="5" spans="1:6">
+      <c r="A5">
         <v>169377692468414</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Estadio de Mendizorroza</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5">
         <v>42.8371</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5">
         <v>-2.6882</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5">
         <v>19840</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5">
         <v>2885</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="n">
+    <row r="6" spans="1:6">
+      <c r="A6">
         <v>153291080865923</v>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Mestalla</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6">
         <v>39.474528</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6">
         <v>-0.358157</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6">
         <v>49430</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6">
         <v>2828</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="n">
+    <row r="7" spans="1:6">
+      <c r="A7">
         <v>214015032212846</v>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Estadio Abanca Balaídos</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7">
         <v>42.211122</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7">
         <v>-8.739231</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7">
         <v>24870</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7">
         <v>2821</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="n">
+    <row r="8" spans="1:6">
+      <c r="A8">
         <v>180874049184635</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>San Mamés</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8">
         <v>43.264204</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8">
         <v>-2.949391</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8">
         <v>53289</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8">
         <v>2825</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="n">
+    <row r="9" spans="1:6">
+      <c r="A9">
         <v>219090305953065</v>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>RCDE Stadium</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9">
         <v>41.347807</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9">
         <v>2.074801</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9">
         <v>40000</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9">
         <v>2814</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="n">
+    <row r="10" spans="1:6">
+      <c r="A10">
         <v>110480584246559</v>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Estadio Martínez Valero</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10">
         <v>38.267044</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10">
         <v>-0.663305</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10">
         <v>31388</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10">
         <v>2846</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="n">
+    <row r="11" spans="1:6">
+      <c r="A11">
         <v>203279944064655</v>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Bernabéu</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11">
         <v>40.453</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11">
         <v>-3.6883</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11">
         <v>84744</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11">
         <v>2829</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="n">
+    <row r="12" spans="1:6">
+      <c r="A12">
         <v>169514417131881</v>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Benito Villamarin</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12">
         <v>37.356535</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12">
         <v>-5.981757</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12">
         <v>60721</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12">
         <v>2816</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="n">
+    <row r="13" spans="1:6">
+      <c r="A13">
         <v>27672874748758</v>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Riyadh Air Metropolitano</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13">
         <v>40.436053</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13">
         <v>-3.599716</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13">
         <v>70460</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13">
         <v>2836</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="n">
+    <row r="14" spans="1:6">
+      <c r="A14">
         <v>104745605050045</v>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Ciudad de Valencia</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
+      <c r="B14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14">
         <v>39.4946</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14">
         <v>-0.3633</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14">
         <v>26354</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14">
         <v>2849</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="n">
+    <row r="15" spans="1:6">
+      <c r="A15">
         <v>82384199862713</v>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Estadio El Sadar</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
+      <c r="B15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15">
         <v>42.796662</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15">
         <v>-1.637131</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15">
         <v>23576</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15">
         <v>2820</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="n">
+    <row r="16" spans="1:6">
+      <c r="A16">
         <v>158255153981266</v>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Reale Arena</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16">
         <v>43.301337</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16">
         <v>-1.973552</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16">
         <v>40000</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16">
         <v>2824</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="n">
+    <row r="17" spans="1:6">
+      <c r="A17">
         <v>153867312518944</v>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Carlos Tartiere</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
+      <c r="B17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17">
         <v>43.360872</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17">
         <v>-5.870332</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17">
         <v>30500</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17">
         <v>2851</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="n">
+    <row r="18" spans="1:6">
+      <c r="A18">
         <v>15578792036393</v>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Ramón Sánchez Pizjuán</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
+      <c r="B18" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18">
         <v>37.384634</v>
       </c>
-      <c r="D18" t="n">
+      <c r="D18">
         <v>-5.971156</v>
       </c>
-      <c r="E18" t="n">
+      <c r="E18">
         <v>42714</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F18">
         <v>2833</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="n">
+    <row r="19" spans="1:6">
+      <c r="A19">
         <v>260618179886907</v>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Estadio de Vallecas</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
+      <c r="B19" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19">
         <v>40.3921</v>
       </c>
-      <c r="D19" t="n">
+      <c r="D19">
         <v>-3.6587</v>
       </c>
-      <c r="E19" t="n">
+      <c r="E19">
         <v>14708</v>
       </c>
-      <c r="F19" t="n">
+      <c r="F19">
         <v>2818</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="n">
+    <row r="20" spans="1:6">
+      <c r="A20">
         <v>206550188571937</v>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Coliseum Alfonso Pérez</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
+      <c r="B20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20">
         <v>40.325725</v>
       </c>
-      <c r="D20" t="n">
+      <c r="D20">
         <v>-3.714933</v>
       </c>
-      <c r="E20" t="n">
+      <c r="E20">
         <v>17393</v>
       </c>
-      <c r="F20" t="n">
+      <c r="F20">
         <v>2859</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="n">
+    <row r="21" spans="1:6">
+      <c r="A21">
         <v>230130911226690</v>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Estadi Johan Cruyff</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
+      <c r="B21" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21">
         <v>41.3742</v>
       </c>
-      <c r="D21" t="n">
+      <c r="D21">
         <v>2.050553</v>
       </c>
-      <c r="E21" t="n">
+      <c r="E21">
         <v>6000</v>
       </c>
-      <c r="F21" t="n">
+      <c r="F21">
         <v>2817</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="n">
+    <row r="22" spans="1:6">
+      <c r="A22">
         <v>157913660528328</v>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Olímpic Lluís Companys</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
+      <c r="B22" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22">
         <v>41.36472</v>
       </c>
-      <c r="D22" t="n">
+      <c r="D22">
         <v>2.155645</v>
       </c>
-      <c r="E22" t="n">
+      <c r="E22">
         <v>55926</v>
       </c>
-      <c r="F22" t="n">
+      <c r="F22">
         <v>2817</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="n">
+    <row r="23" spans="1:6">
+      <c r="A23">
         <v>170718495619227</v>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Estadio de la Cartuja</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
+      <c r="B23" t="s">
+        <v>27</v>
+      </c>
+      <c r="C23">
         <v>37.417235</v>
       </c>
-      <c r="D23" t="n">
+      <c r="D23">
         <v>-6.004613</v>
       </c>
-      <c r="E23" t="n">
+      <c r="E23">
         <v>70000</v>
       </c>
-      <c r="F23" t="n">
+      <c r="F23">
         <v>2816</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="n">
+    <row r="24" spans="1:6">
+      <c r="A24">
         <v>77066563565456</v>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Spotify Camp Nou</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
+      <c r="B24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24">
         <v>41.380881</v>
       </c>
-      <c r="D24" t="n">
+      <c r="D24">
         <v>2.122818</v>
       </c>
-      <c r="E24" t="n">
+      <c r="E24">
         <v>45401</v>
       </c>
-      <c r="F24" t="n">
+      <c r="F24">
         <v>2817</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
imlemented matchs and venues
</commit_message>
<xml_diff>
--- a/webscrapping/sofascore/Server/files_initted/estadios_info_db.xlsx
+++ b/webscrapping/sofascore/Server/files_initted/estadios_info_db.xlsx
@@ -1,132 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
-  <si>
-    <t>id_estadio</t>
-  </si>
-  <si>
-    <t>nombre</t>
-  </si>
-  <si>
-    <t>latitud</t>
-  </si>
-  <si>
-    <t>longitud</t>
-  </si>
-  <si>
-    <t>capacidad</t>
-  </si>
-  <si>
-    <t>id_equipo</t>
-  </si>
-  <si>
-    <t>Estadi Montilivi</t>
-  </si>
-  <si>
-    <t>Estadio de la Ceramica</t>
-  </si>
-  <si>
-    <t>Estadi de Son Moix</t>
-  </si>
-  <si>
-    <t>Estadio de Mendizorroza</t>
-  </si>
-  <si>
-    <t>Mestalla</t>
-  </si>
-  <si>
-    <t>Estadio Abanca Balaídos</t>
-  </si>
-  <si>
-    <t>San Mamés</t>
-  </si>
-  <si>
-    <t>RCDE Stadium</t>
-  </si>
-  <si>
-    <t>Estadio Martínez Valero</t>
-  </si>
-  <si>
-    <t>Bernabéu</t>
-  </si>
-  <si>
-    <t>Benito Villamarin</t>
-  </si>
-  <si>
-    <t>Riyadh Air Metropolitano</t>
-  </si>
-  <si>
-    <t>Ciudad de Valencia</t>
-  </si>
-  <si>
-    <t>Estadio El Sadar</t>
-  </si>
-  <si>
-    <t>Reale Arena</t>
-  </si>
-  <si>
-    <t>Carlos Tartiere</t>
-  </si>
-  <si>
-    <t>Ramón Sánchez Pizjuán</t>
-  </si>
-  <si>
-    <t>Estadio de Vallecas</t>
-  </si>
-  <si>
-    <t>Coliseum Alfonso Pérez</t>
-  </si>
-  <si>
-    <t>Estadi Johan Cruyff</t>
-  </si>
-  <si>
-    <t>Olímpic Lluís Companys</t>
-  </si>
-  <si>
-    <t>Estadio de la Cartuja</t>
-  </si>
-  <si>
-    <t>Spotify Camp Nou</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -141,35 +46,93 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -457,491 +420,553 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F24"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id_estadio</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>nombre</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>latitud</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>longitud</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>capacidad</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>id_equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
         <v>260827297577701</v>
       </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Estadi Montilivi</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>41.9611</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>2.8278</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="n">
         <v>14624</v>
       </c>
-      <c r="F2">
+      <c r="F2" t="n">
         <v>24264</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
-      <c r="A3">
+    <row r="3">
+      <c r="A3" t="n">
         <v>190203353926090</v>
       </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Estadio de la Ceramica</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>39.944208</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>-0.103405</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="n">
         <v>23500</v>
       </c>
-      <c r="F3">
+      <c r="F3" t="n">
         <v>2819</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
-      <c r="A4">
+    <row r="4">
+      <c r="A4" t="n">
         <v>99680602019422</v>
       </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Estadi de Son Moix</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>39.589935</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>2.630116</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="n">
         <v>26020</v>
       </c>
-      <c r="F4">
+      <c r="F4" t="n">
         <v>2826</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
-      <c r="A5">
+    <row r="5">
+      <c r="A5" t="n">
         <v>169377692468414</v>
       </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Estadio de Mendizorroza</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
         <v>42.8371</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>-2.6882</v>
       </c>
-      <c r="E5">
+      <c r="E5" t="n">
         <v>19840</v>
       </c>
-      <c r="F5">
+      <c r="F5" t="n">
         <v>2885</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
-      <c r="A6">
+    <row r="6">
+      <c r="A6" t="n">
         <v>153291080865923</v>
       </c>
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mestalla</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
         <v>39.474528</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>-0.358157</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="n">
         <v>49430</v>
       </c>
-      <c r="F6">
+      <c r="F6" t="n">
         <v>2828</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
-      <c r="A7">
+    <row r="7">
+      <c r="A7" t="n">
         <v>214015032212846</v>
       </c>
-      <c r="B7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Estadio Abanca Balaídos</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
         <v>42.211122</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="n">
         <v>-8.739231</v>
       </c>
-      <c r="E7">
+      <c r="E7" t="n">
         <v>24870</v>
       </c>
-      <c r="F7">
+      <c r="F7" t="n">
         <v>2821</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
-      <c r="A8">
+    <row r="8">
+      <c r="A8" t="n">
         <v>180874049184635</v>
       </c>
-      <c r="B8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>San Mamés</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
         <v>43.264204</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="n">
         <v>-2.949391</v>
       </c>
-      <c r="E8">
+      <c r="E8" t="n">
         <v>53289</v>
       </c>
-      <c r="F8">
+      <c r="F8" t="n">
         <v>2825</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
-      <c r="A9">
+    <row r="9">
+      <c r="A9" t="n">
         <v>219090305953065</v>
       </c>
-      <c r="B9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>RCDE Stadium</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
         <v>41.347807</v>
       </c>
-      <c r="D9">
+      <c r="D9" t="n">
         <v>2.074801</v>
       </c>
-      <c r="E9">
+      <c r="E9" t="n">
         <v>40000</v>
       </c>
-      <c r="F9">
+      <c r="F9" t="n">
         <v>2814</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
-      <c r="A10">
+    <row r="10">
+      <c r="A10" t="n">
         <v>110480584246559</v>
       </c>
-      <c r="B10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Estadio Martínez Valero</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
         <v>38.267044</v>
       </c>
-      <c r="D10">
+      <c r="D10" t="n">
         <v>-0.663305</v>
       </c>
-      <c r="E10">
+      <c r="E10" t="n">
         <v>31388</v>
       </c>
-      <c r="F10">
+      <c r="F10" t="n">
         <v>2846</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
-      <c r="A11">
+    <row r="11">
+      <c r="A11" t="n">
         <v>203279944064655</v>
       </c>
-      <c r="B11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Bernabéu</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
         <v>40.453</v>
       </c>
-      <c r="D11">
+      <c r="D11" t="n">
         <v>-3.6883</v>
       </c>
-      <c r="E11">
+      <c r="E11" t="n">
         <v>84744</v>
       </c>
-      <c r="F11">
+      <c r="F11" t="n">
         <v>2829</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
-      <c r="A12">
+    <row r="12">
+      <c r="A12" t="n">
         <v>169514417131881</v>
       </c>
-      <c r="B12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Benito Villamarin</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
         <v>37.356535</v>
       </c>
-      <c r="D12">
+      <c r="D12" t="n">
         <v>-5.981757</v>
       </c>
-      <c r="E12">
+      <c r="E12" t="n">
         <v>60721</v>
       </c>
-      <c r="F12">
+      <c r="F12" t="n">
         <v>2816</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
-      <c r="A13">
+    <row r="13">
+      <c r="A13" t="n">
         <v>27672874748758</v>
       </c>
-      <c r="B13" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Riyadh Air Metropolitano</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
         <v>40.436053</v>
       </c>
-      <c r="D13">
+      <c r="D13" t="n">
         <v>-3.599716</v>
       </c>
-      <c r="E13">
+      <c r="E13" t="n">
         <v>70460</v>
       </c>
-      <c r="F13">
+      <c r="F13" t="n">
         <v>2836</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
-      <c r="A14">
+    <row r="14">
+      <c r="A14" t="n">
         <v>104745605050045</v>
       </c>
-      <c r="B14" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Ciudad de Valencia</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
         <v>39.4946</v>
       </c>
-      <c r="D14">
+      <c r="D14" t="n">
         <v>-0.3633</v>
       </c>
-      <c r="E14">
+      <c r="E14" t="n">
         <v>26354</v>
       </c>
-      <c r="F14">
+      <c r="F14" t="n">
         <v>2849</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
-      <c r="A15">
+    <row r="15">
+      <c r="A15" t="n">
         <v>82384199862713</v>
       </c>
-      <c r="B15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Estadio El Sadar</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
         <v>42.796662</v>
       </c>
-      <c r="D15">
+      <c r="D15" t="n">
         <v>-1.637131</v>
       </c>
-      <c r="E15">
+      <c r="E15" t="n">
         <v>23576</v>
       </c>
-      <c r="F15">
+      <c r="F15" t="n">
         <v>2820</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
-      <c r="A16">
+    <row r="16">
+      <c r="A16" t="n">
         <v>158255153981266</v>
       </c>
-      <c r="B16" t="s">
-        <v>20</v>
-      </c>
-      <c r="C16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Reale Arena</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
         <v>43.301337</v>
       </c>
-      <c r="D16">
+      <c r="D16" t="n">
         <v>-1.973552</v>
       </c>
-      <c r="E16">
+      <c r="E16" t="n">
         <v>40000</v>
       </c>
-      <c r="F16">
+      <c r="F16" t="n">
         <v>2824</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
-      <c r="A17">
+    <row r="17">
+      <c r="A17" t="n">
         <v>153867312518944</v>
       </c>
-      <c r="B17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Carlos Tartiere</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
         <v>43.360872</v>
       </c>
-      <c r="D17">
+      <c r="D17" t="n">
         <v>-5.870332</v>
       </c>
-      <c r="E17">
+      <c r="E17" t="n">
         <v>30500</v>
       </c>
-      <c r="F17">
+      <c r="F17" t="n">
         <v>2851</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
-      <c r="A18">
+    <row r="18">
+      <c r="A18" t="n">
         <v>15578792036393</v>
       </c>
-      <c r="B18" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Ramón Sánchez Pizjuán</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
         <v>37.384634</v>
       </c>
-      <c r="D18">
+      <c r="D18" t="n">
         <v>-5.971156</v>
       </c>
-      <c r="E18">
+      <c r="E18" t="n">
         <v>42714</v>
       </c>
-      <c r="F18">
+      <c r="F18" t="n">
         <v>2833</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
-      <c r="A19">
+    <row r="19">
+      <c r="A19" t="n">
         <v>260618179886907</v>
       </c>
-      <c r="B19" t="s">
-        <v>23</v>
-      </c>
-      <c r="C19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Estadio de Vallecas</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
         <v>40.3921</v>
       </c>
-      <c r="D19">
+      <c r="D19" t="n">
         <v>-3.6587</v>
       </c>
-      <c r="E19">
+      <c r="E19" t="n">
         <v>14708</v>
       </c>
-      <c r="F19">
+      <c r="F19" t="n">
         <v>2818</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
-      <c r="A20">
+    <row r="20">
+      <c r="A20" t="n">
         <v>206550188571937</v>
       </c>
-      <c r="B20" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Coliseum Alfonso Pérez</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
         <v>40.325725</v>
       </c>
-      <c r="D20">
+      <c r="D20" t="n">
         <v>-3.714933</v>
       </c>
-      <c r="E20">
+      <c r="E20" t="n">
         <v>17393</v>
       </c>
-      <c r="F20">
+      <c r="F20" t="n">
         <v>2859</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
-      <c r="A21">
+    <row r="21">
+      <c r="A21" t="n">
         <v>230130911226690</v>
       </c>
-      <c r="B21" t="s">
-        <v>25</v>
-      </c>
-      <c r="C21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Estadi Johan Cruyff</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
         <v>41.3742</v>
       </c>
-      <c r="D21">
+      <c r="D21" t="n">
         <v>2.050553</v>
       </c>
-      <c r="E21">
+      <c r="E21" t="n">
         <v>6000</v>
       </c>
-      <c r="F21">
+      <c r="F21" t="n">
         <v>2817</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
-      <c r="A22">
+    <row r="22">
+      <c r="A22" t="n">
         <v>157913660528328</v>
       </c>
-      <c r="B22" t="s">
-        <v>26</v>
-      </c>
-      <c r="C22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Olímpic Lluís Companys</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
         <v>41.36472</v>
       </c>
-      <c r="D22">
+      <c r="D22" t="n">
         <v>2.155645</v>
       </c>
-      <c r="E22">
+      <c r="E22" t="n">
         <v>55926</v>
       </c>
-      <c r="F22">
+      <c r="F22" t="n">
         <v>2817</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
-      <c r="A23">
+    <row r="23">
+      <c r="A23" t="n">
         <v>170718495619227</v>
       </c>
-      <c r="B23" t="s">
-        <v>27</v>
-      </c>
-      <c r="C23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Estadio de la Cartuja</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
         <v>37.417235</v>
       </c>
-      <c r="D23">
+      <c r="D23" t="n">
         <v>-6.004613</v>
       </c>
-      <c r="E23">
+      <c r="E23" t="n">
         <v>70000</v>
       </c>
-      <c r="F23">
+      <c r="F23" t="n">
         <v>2816</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
-      <c r="A24">
+    <row r="24">
+      <c r="A24" t="n">
         <v>77066563565456</v>
       </c>
-      <c r="B24" t="s">
-        <v>28</v>
-      </c>
-      <c r="C24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Spotify Camp Nou</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
         <v>41.380881</v>
       </c>
-      <c r="D24">
+      <c r="D24" t="n">
         <v>2.122818</v>
       </c>
-      <c r="E24">
+      <c r="E24" t="n">
         <v>45401</v>
       </c>
-      <c r="F24">
+      <c r="F24" t="n">
         <v>2817</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
implemented filters for both matches and rankings
</commit_message>
<xml_diff>
--- a/webscrapping/sofascore/Server/files_initted/estadios_info_db.xlsx
+++ b/webscrapping/sofascore/Server/files_initted/estadios_info_db.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="44">
   <si>
     <t>id_estadio</t>
   </si>
@@ -112,7 +112,7 @@
     <t>Vila-real, la Plana Baixa, Castelló / Castellón, Valencian Community, 12540, Spain</t>
   </si>
   <si>
-    <t>Palma de Mallorca, Balearic Islands, Spain</t>
+    <t>Desconocido</t>
   </si>
   <si>
     <t>Vitoria-Gasteiz, Gasteizko kuadrilla/Cuadrilla de Vitoria, Álava, Autonomous Community of the Basque Country, Spain</t>
@@ -121,28 +121,19 @@
     <t>Valencia, Comarca de València, Valencia, Valencian Community, Spain</t>
   </si>
   <si>
-    <t>Vigo, Pontevedra, Galicia, Spain</t>
-  </si>
-  <si>
     <t>Bilbao, Biscay, Autonomous Community of the Basque Country, Spain</t>
   </si>
   <si>
     <t>Cornellà de Llobregat, Baix Llobregat, Barcelona, Catalonia, 08940, Spain</t>
   </si>
   <si>
-    <t>Elx / Elche, el Baix Vinalopó, Alacant / Alicante, Valencian Community, Spain</t>
-  </si>
-  <si>
     <t>Madrid, Community of Madrid, Spain</t>
   </si>
   <si>
     <t>Seville, Sevilla, Andalusia, Spain</t>
   </si>
   <si>
-    <t>Desconocido</t>
-  </si>
-  <si>
-    <t>Pamplona, Iruñerria / Comarca de Pamplona, Navarre, Spain</t>
+    <t>San Sebastián, Gipuzkoa, Autonomous Community of the Basque Country, Spain</t>
   </si>
   <si>
     <t>Oviedo, Asturias, Spain</t>
@@ -155,9 +146,6 @@
   </si>
   <si>
     <t>Barcelona, Barcelonès, Barcelona, Catalonia, Spain</t>
-  </si>
-  <si>
-    <t>Santiponce, Sevilla, Andalusia, 41970, Spain</t>
   </si>
 </sst>
 </file>
@@ -670,7 +658,7 @@
         <v>-8.739231</v>
       </c>
       <c r="E7" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F7">
         <v>24870</v>
@@ -693,7 +681,7 @@
         <v>-2.949391</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F8">
         <v>53289</v>
@@ -716,7 +704,7 @@
         <v>2.074801</v>
       </c>
       <c r="E9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F9">
         <v>40000</v>
@@ -739,7 +727,7 @@
         <v>-0.663305</v>
       </c>
       <c r="E10" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F10">
         <v>31388</v>
@@ -762,7 +750,7 @@
         <v>-3.6883</v>
       </c>
       <c r="E11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F11">
         <v>84744</v>
@@ -785,7 +773,7 @@
         <v>-5.981757</v>
       </c>
       <c r="E12" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F12">
         <v>60721</v>
@@ -808,7 +796,7 @@
         <v>-3.599716</v>
       </c>
       <c r="E13" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F13">
         <v>70460</v>
@@ -854,7 +842,7 @@
         <v>-1.637131</v>
       </c>
       <c r="E15" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="F15">
         <v>23576</v>
@@ -877,7 +865,7 @@
         <v>-1.973552</v>
       </c>
       <c r="E16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F16">
         <v>40000</v>
@@ -900,7 +888,7 @@
         <v>-5.870332</v>
       </c>
       <c r="E17" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F17">
         <v>30500</v>
@@ -923,7 +911,7 @@
         <v>-5.971156</v>
       </c>
       <c r="E18" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="F18">
         <v>42714</v>
@@ -946,7 +934,7 @@
         <v>-3.6587</v>
       </c>
       <c r="E19" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F19">
         <v>14708</v>
@@ -969,7 +957,7 @@
         <v>-3.714933</v>
       </c>
       <c r="E20" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F20">
         <v>17393</v>
@@ -992,7 +980,7 @@
         <v>2.050553</v>
       </c>
       <c r="E21" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F21">
         <v>6000</v>
@@ -1015,7 +1003,7 @@
         <v>2.155645</v>
       </c>
       <c r="E22" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F22">
         <v>55926</v>
@@ -1038,7 +1026,7 @@
         <v>-6.004613</v>
       </c>
       <c r="E23" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="F23">
         <v>70000</v>
@@ -1061,7 +1049,7 @@
         <v>2.122818</v>
       </c>
       <c r="E24" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F24">
         <v>45401</v>

</xml_diff>